<commit_message>
#11 JLCPCB BOM Updated extra Centroid File Folder Deleted
</commit_message>
<xml_diff>
--- a/Design Files/Catan_Board/Master_PCB/BOM/JLCPCB BOM.xlsx
+++ b/Design Files/Catan_Board/Master_PCB/BOM/JLCPCB BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="183">
   <si>
     <t>Comment</t>
   </si>
@@ -54,6 +54,9 @@
     <t>560uF</t>
   </si>
   <si>
+    <t>100uF</t>
+  </si>
+  <si>
     <t>1nF</t>
   </si>
   <si>
@@ -108,7 +111,7 @@
     <t>1K</t>
   </si>
   <si>
-    <t>3.01K</t>
+    <t>1.54k</t>
   </si>
   <si>
     <t>10K</t>
@@ -135,6 +138,9 @@
     <t>390R</t>
   </si>
   <si>
+    <t>50K</t>
+  </si>
+  <si>
     <t>B3U-1000P</t>
   </si>
   <si>
@@ -201,6 +207,9 @@
     <t>C37</t>
   </si>
   <si>
+    <t>C38</t>
+  </si>
+  <si>
     <t>C41, C55</t>
   </si>
   <si>
@@ -252,7 +261,7 @@
     <t>R2, R6, R10</t>
   </si>
   <si>
-    <t>R3, R4</t>
+    <t>R3</t>
   </si>
   <si>
     <t>R5, R7, R8, R14, R15, R16, R20, R21, R22, R23, R24, R25, R27, R28, R29</t>
@@ -282,6 +291,9 @@
     <t>R30</t>
   </si>
   <si>
+    <t>R31</t>
+  </si>
+  <si>
     <t>SW1</t>
   </si>
   <si>
@@ -330,6 +342,9 @@
     <t>EEEFN1V561UP</t>
   </si>
   <si>
+    <t>Cap-1206</t>
+  </si>
+  <si>
     <t>CAP-0603</t>
   </si>
   <si>
@@ -372,6 +387,9 @@
     <t>Res-0603</t>
   </si>
   <si>
+    <t>Res-0402</t>
+  </si>
+  <si>
     <t>TQFN-16-EP(4x4)_</t>
   </si>
   <si>
@@ -486,7 +504,7 @@
     <t>C165964</t>
   </si>
   <si>
-    <t>C278616</t>
+    <t>C396136</t>
   </si>
   <si>
     <t>C140867</t>
@@ -513,6 +531,9 @@
     <t>C137632</t>
   </si>
   <si>
+    <t>C2073717</t>
+  </si>
+  <si>
     <t>C231329</t>
   </si>
   <si>
@@ -538,6 +559,9 @@
   </si>
   <si>
     <t>C115962</t>
+  </si>
+  <si>
+    <t>C2167823</t>
   </si>
   <si>
     <t>C69679</t>
@@ -989,7 +1013,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1003,13 +1027,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1017,13 +1041,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="36" x14ac:dyDescent="0.25">
@@ -1031,13 +1055,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1045,13 +1069,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1059,13 +1083,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1073,13 +1097,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1087,13 +1111,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1101,13 +1125,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1115,13 +1139,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1129,13 +1153,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1143,13 +1167,13 @@
         <v>3</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1157,13 +1181,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1171,13 +1195,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1185,13 +1209,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>138</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1199,13 +1223,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1213,13 +1237,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1227,13 +1251,13 @@
         <v>14</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1241,13 +1265,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>173</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1255,13 +1279,13 @@
         <v>16</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>142</v>
+        <v>181</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1269,13 +1293,13 @@
         <v>17</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C20" s="5">
-        <v>1051330011</v>
+        <v>68</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>113</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1283,55 +1307,55 @@
         <v>18</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>109</v>
+        <v>69</v>
+      </c>
+      <c r="C21" s="7">
+        <v>1051330011</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
-        <v>20</v>
+      <c r="A22" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>174</v>
+        <v>70</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>20</v>
+        <v>114</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4">
+      <c r="A23" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="6">
         <v>22284020</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>21</v>
-      </c>
       <c r="B24" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1339,13 +1363,13 @@
         <v>22</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1353,13 +1377,13 @@
         <v>23</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1367,27 +1391,27 @@
         <v>24</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>151</v>
+      <c r="B28" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1395,13 +1419,13 @@
         <v>26</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1409,13 +1433,13 @@
         <v>27</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1423,13 +1447,13 @@
         <v>28</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1437,41 +1461,41 @@
         <v>29</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1479,13 +1503,13 @@
         <v>32</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1493,13 +1517,13 @@
         <v>33</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1507,41 +1531,41 @@
         <v>34</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1549,13 +1573,13 @@
         <v>36</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1563,13 +1587,13 @@
         <v>37</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1577,13 +1601,13 @@
         <v>38</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>38</v>
+        <v>121</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1591,13 +1615,13 @@
         <v>39</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1605,13 +1629,13 @@
         <v>40</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>118</v>
+        <v>40</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1619,13 +1643,13 @@
         <v>41</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -1633,13 +1657,13 @@
         <v>42</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1647,13 +1671,13 @@
         <v>43</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1661,13 +1685,13 @@
         <v>44</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1675,13 +1699,13 @@
         <v>45</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1689,13 +1713,41 @@
         <v>46</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>172</v>
+        <v>177</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
C37 part number updated #13
</commit_message>
<xml_diff>
--- a/Design Files/Catan_Board/Master_PCB/BOM/JLCPCB BOM.xlsx
+++ b/Design Files/Catan_Board/Master_PCB/BOM/JLCPCB BOM.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\jakekrum-catanboard\Design Files\Catan_Board\Master_PCB\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Faizan\GitHub\jakekrum-catanboard\Design Files\Catan_Board\Master_PCB\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB56753B-FF78-4D85-9DA5-A6AB69DAA2C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -339,9 +340,6 @@
     <t>UUD1A102MNL1GS</t>
   </si>
   <si>
-    <t>EEEFN1V561UP</t>
-  </si>
-  <si>
     <t>Cap-1206</t>
   </si>
   <si>
@@ -450,9 +448,6 @@
     <t>C445277</t>
   </si>
   <si>
-    <t>C494848</t>
-  </si>
-  <si>
     <t>C309470</t>
   </si>
   <si>
@@ -568,12 +563,18 @@
   </si>
   <si>
     <t>J12, J13</t>
+  </si>
+  <si>
+    <t>GVT1C561M0810</t>
+  </si>
+  <si>
+    <t>C2980166</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1011,18 +1012,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:D52"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1033,10 +1034,10 @@
         <v>100</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1047,10 +1048,10 @@
         <v>101</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="36" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="36" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -1061,10 +1062,10 @@
         <v>102</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
@@ -1075,10 +1076,10 @@
         <v>102</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -1089,10 +1090,10 @@
         <v>102</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
@@ -1103,10 +1104,10 @@
         <v>103</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
@@ -1117,10 +1118,10 @@
         <v>102</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
@@ -1131,10 +1132,10 @@
         <v>102</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -1145,10 +1146,10 @@
         <v>102</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>8</v>
       </c>
@@ -1159,10 +1160,10 @@
         <v>102</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>3</v>
       </c>
@@ -1173,10 +1174,10 @@
         <v>104</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
@@ -1187,10 +1188,10 @@
         <v>105</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>10</v>
       </c>
@@ -1198,13 +1199,13 @@
         <v>61</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>106</v>
+        <v>181</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>11</v>
       </c>
@@ -1212,13 +1213,13 @@
         <v>62</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>12</v>
       </c>
@@ -1226,13 +1227,13 @@
         <v>63</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>13</v>
       </c>
@@ -1240,13 +1241,13 @@
         <v>64</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>14</v>
       </c>
@@ -1254,13 +1255,13 @@
         <v>65</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>15</v>
       </c>
@@ -1268,13 +1269,13 @@
         <v>66</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>16</v>
       </c>
@@ -1282,13 +1283,13 @@
         <v>67</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>17</v>
       </c>
@@ -1296,13 +1297,13 @@
         <v>68</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>18</v>
       </c>
@@ -1313,10 +1314,10 @@
         <v>1051330011</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>19</v>
       </c>
@@ -1324,27 +1325,27 @@
         <v>70</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="6">
         <v>22284020</v>
       </c>
@@ -1352,13 +1353,13 @@
         <v>71</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>22</v>
       </c>
@@ -1366,13 +1367,13 @@
         <v>72</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>23</v>
       </c>
@@ -1380,13 +1381,13 @@
         <v>73</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>24</v>
       </c>
@@ -1394,13 +1395,13 @@
         <v>74</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>25</v>
       </c>
@@ -1408,13 +1409,13 @@
         <v>75</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>26</v>
       </c>
@@ -1422,13 +1423,13 @@
         <v>76</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>27</v>
       </c>
@@ -1436,13 +1437,13 @@
         <v>77</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>28</v>
       </c>
@@ -1450,13 +1451,13 @@
         <v>78</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>29</v>
       </c>
@@ -1464,13 +1465,13 @@
         <v>79</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>30</v>
       </c>
@@ -1478,13 +1479,13 @@
         <v>80</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="24" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>31</v>
       </c>
@@ -1492,13 +1493,13 @@
         <v>81</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>32</v>
       </c>
@@ -1506,13 +1507,13 @@
         <v>82</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>33</v>
       </c>
@@ -1520,13 +1521,13 @@
         <v>83</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>34</v>
       </c>
@@ -1534,13 +1535,13 @@
         <v>84</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>35</v>
       </c>
@@ -1548,13 +1549,13 @@
         <v>85</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>20</v>
       </c>
@@ -1562,13 +1563,13 @@
         <v>86</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>36</v>
       </c>
@@ -1576,13 +1577,13 @@
         <v>87</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>37</v>
       </c>
@@ -1590,13 +1591,13 @@
         <v>88</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>38</v>
       </c>
@@ -1604,13 +1605,13 @@
         <v>89</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>39</v>
       </c>
@@ -1618,13 +1619,13 @@
         <v>90</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>40</v>
       </c>
@@ -1635,10 +1636,10 @@
         <v>40</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>41</v>
       </c>
@@ -1646,13 +1647,13 @@
         <v>92</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>42</v>
       </c>
@@ -1660,13 +1661,13 @@
         <v>93</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>43</v>
       </c>
@@ -1674,13 +1675,13 @@
         <v>94</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>44</v>
       </c>
@@ -1688,13 +1689,13 @@
         <v>95</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>45</v>
       </c>
@@ -1702,13 +1703,13 @@
         <v>96</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>46</v>
       </c>
@@ -1716,13 +1717,13 @@
         <v>97</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
         <v>47</v>
       </c>
@@ -1730,13 +1731,13 @@
         <v>98</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>48</v>
       </c>
@@ -1744,10 +1745,10 @@
         <v>99</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>